<commit_message>
Dashboard update 2026-08-09 21:05
</commit_message>
<xml_diff>
--- a/excel/Indemo.xlsx
+++ b/excel/Indemo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Investavimas 2026.06.03\Indemo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evald\OneDrive\Dokumentai\portfolio-analytics\portfolio-dashboard-clean\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E406AABB-EAB9-4F79-9F0C-F9D035EDD623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4954635D-AEF7-4308-AA48-64F8A3D53787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="33" r:id="rId1"/>
@@ -7363,7 +7363,7 @@
       </c>
       <c r="T3" s="6">
         <f ca="1">XIRR(Pinigai!K2:K200,Pinigai!A2:A200)</f>
-        <v>0.14429696202278133</v>
+        <v>0.14164766669273374</v>
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.25">
@@ -17249,7 +17249,7 @@
       </c>
       <c r="I2" s="6">
         <f ca="1">XIRR(K2:K200,A2:A200)</f>
-        <v>0.14429696202278133</v>
+        <v>0.14164766669273374</v>
       </c>
       <c r="J2" s="13"/>
       <c r="K2" s="5">
@@ -18951,7 +18951,7 @@
     <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200" s="24">
         <f ca="1">TODAY()</f>
-        <v>46236</v>
+        <v>46243</v>
       </c>
       <c r="B200" s="26"/>
       <c r="C200" s="26"/>

</xml_diff>